<commit_message>
Modified Browser class to Run pipelines manually.
</commit_message>
<xml_diff>
--- a/excel/186880.xlsx
+++ b/excel/186880.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Selenium with Java Learnings\eclipse-workspace (1)\eclipse-workspace\ChorusAutomation\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B4482F3-B252-48A1-B7E8-5A81948A6638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439B7AD1-44E8-4CFD-9D67-05925F5A4D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
   <si>
     <t>Project</t>
   </si>
@@ -202,12 +202,18 @@
       <t>, regardless of the original filename length.</t>
     </r>
   </si>
+  <si>
+    <t>31 December 2025</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="[$-24009]mmmm\ dd\,\ yyyy;@"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -248,6 +254,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -348,14 +360,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -812,7 +824,7 @@
       <c r="J2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="13" t="s">
         <v>30</v>
       </c>
       <c r="L2" s="3"/>
@@ -827,7 +839,7 @@
         <v>27</v>
       </c>
       <c r="Q2" s="3"/>
-      <c r="R2" s="12"/>
+      <c r="R2" s="11"/>
       <c r="S2" s="1" t="s">
         <v>31</v>
       </c>
@@ -845,7 +857,7 @@
       <c r="B3" s="10">
         <v>2</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>34</v>
       </c>
       <c r="D3" s="3" t="s">
@@ -860,7 +872,7 @@
       <c r="G3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="12" t="s">
         <v>34</v>
       </c>
       <c r="I3" s="3">
@@ -869,8 +881,8 @@
       <c r="J3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="11" t="s">
-        <v>30</v>
+      <c r="K3" s="13" t="s">
+        <v>38</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3" t="s">
@@ -884,7 +896,7 @@
         <v>27</v>
       </c>
       <c r="Q3" s="3"/>
-      <c r="R3" s="12"/>
+      <c r="R3" s="11"/>
       <c r="S3" s="1" t="s">
         <v>35</v>
       </c>
@@ -896,29 +908,13 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="45ca309a-9f07-4f68-80cb-ee78bcc0241f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004B66CC44786BB0439F8987298B7E9A0C" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f2f484eec5e1492443c87c6cfef49cde">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="45ca309a-9f07-4f68-80cb-ee78bcc0241f" xmlns:ns4="f9f82460-e327-4066-9827-168a447f3884" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f98e04737e4923a0a8240dd31c51e3f" ns3:_="" ns4:_="">
     <xsd:import namespace="45ca309a-9f07-4f68-80cb-ee78bcc0241f"/>
@@ -1151,25 +1147,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A2A915A-FEC9-4A8C-8682-D88E304B19B0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="45ca309a-9f07-4f68-80cb-ee78bcc0241f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70C273EC-3505-4825-9E03-C17F1892B777}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="45ca309a-9f07-4f68-80cb-ee78bcc0241f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5766244B-F4F7-43F8-9E74-49A9A3F6942A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1186,4 +1181,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70C273EC-3505-4825-9E03-C17F1892B777}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="45ca309a-9f07-4f68-80cb-ee78bcc0241f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A2A915A-FEC9-4A8C-8682-D88E304B19B0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>